<commit_message>
docs: clarify default input values for PIM boundary cases
</commit_message>
<xml_diff>
--- a/docs/test-cases/members/Group01_23130226_VoMinhNhut.xlsx
+++ b/docs/test-cases/members/Group01_23130226_VoMinhNhut.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rde46881891a9440f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test case List" sheetId="2" r:id="Re227121ff27a4cfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestDesign" sheetId="3" r:id="R7b5cfd126cef4463"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_EMP" sheetId="4" r:id="Rfa51bb0840524cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_PERSONAL" sheetId="5" r:id="R34ed9c7be1b84e20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_JOB" sheetId="6" r:id="R4456e1d9b5aa4ced"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data" sheetId="7" r:id="Rd858ca0f510241c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Plan" sheetId="8" r:id="R8c412de4fab34473"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="9" r:id="R417b1d9d9ad4456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R739b45e188bb48db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test case List" sheetId="2" r:id="R9ac2463c9267459f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestDesign" sheetId="3" r:id="Ra7589f21bff5486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_EMP" sheetId="4" r:id="R588a0c4c3ae041d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_PERSONAL" sheetId="5" r:id="Ra576c08c4f93428c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_JOB" sheetId="6" r:id="Re87b1e7ac9514a89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data" sheetId="7" r:id="R3b7c9d1b71d4489e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Plan" sheetId="8" r:id="R58677b5b5fa74174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="9" r:id="Rfd03dbf4708d45ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -189,7 +189,7 @@
         <x:color rgb="FF20603A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE7F2E8"/>
         </x:patternFill>
       </x:fill>
@@ -200,7 +200,7 @@
         <x:color rgb="FFA52323"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -211,7 +211,7 @@
         <x:color rgb="FF805A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -222,7 +222,7 @@
         <x:color rgb="FF525E6D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECEFF3"/>
         </x:patternFill>
       </x:fill>
@@ -233,7 +233,7 @@
         <x:color rgb="FF20603A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE7F2E8"/>
         </x:patternFill>
       </x:fill>
@@ -244,7 +244,7 @@
         <x:color rgb="FFA52323"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -255,7 +255,7 @@
         <x:color rgb="FF805A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -266,7 +266,7 @@
         <x:color rgb="FF525E6D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECEFF3"/>
         </x:patternFill>
       </x:fill>
@@ -277,7 +277,7 @@
         <x:color rgb="FF20603A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE7F2E8"/>
         </x:patternFill>
       </x:fill>
@@ -288,7 +288,7 @@
         <x:color rgb="FFA52323"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -299,7 +299,7 @@
         <x:color rgb="FF805A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -310,7 +310,7 @@
         <x:color rgb="FF525E6D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECEFF3"/>
         </x:patternFill>
       </x:fill>
@@ -4773,13 +4773,25 @@
         <x:v>Kiểm thử chức năng, không scan bảo mật hay load test.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="3"/>
-      <x:c r="B25" s="3"/>
-      <x:c r="C25" s="3"/>
-      <x:c r="D25" s="3"/>
-      <x:c r="E25" s="3"/>
-      <x:c r="F25" s="3"/>
+    <x:row r="25" ht="110" customHeight="1">
+      <x:c r="A25" s="3" t="str">
+        <x:v>ADD_DEFAULT</x:v>
+      </x:c>
+      <x:c r="B25" s="3" t="str">
+        <x:v>First=G01N01; Middle=Minh; Last=NhutBaseline</x:v>
+      </x:c>
+      <x:c r="C25" s="3" t="str">
+        <x:v>Áp dụng cho các ô tên còn lại khi TC chỉ thay một trường hoặc ghi tên hợp lệ. Employee Id dùng ID riêng được chỉ rõ trong TC; nếu chưa chỉ rõ, giữ ID tự sinh và kiểm tra chưa tồn tại.</x:v>
+      </x:c>
+      <x:c r="D25" s="3" t="str">
+        <x:v>Add Employee: chuỗi biên, ID, ảnh và validation</x:v>
+      </x:c>
+      <x:c r="E25" s="3" t="str">
+        <x:v>Sau case, xóa riêng nhân viên đã tạo sau khi giữ bằng chứng.</x:v>
+      </x:c>
+      <x:c r="F25" s="3" t="str">
+        <x:v>Giá trị nêu riêng trong TC được ưu tiên.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="3"/>

</xml_diff>

<commit_message>
docs: align PIM workbook with nhut branch and personal tool choice
</commit_message>
<xml_diff>
--- a/docs/test-cases/members/Group01_23130226_VoMinhNhut.xlsx
+++ b/docs/test-cases/members/Group01_23130226_VoMinhNhut.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R739b45e188bb48db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test case List" sheetId="2" r:id="R9ac2463c9267459f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestDesign" sheetId="3" r:id="Ra7589f21bff5486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_EMP" sheetId="4" r:id="R588a0c4c3ae041d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_PERSONAL" sheetId="5" r:id="Ra576c08c4f93428c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_JOB" sheetId="6" r:id="Re87b1e7ac9514a89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data" sheetId="7" r:id="R3b7c9d1b71d4489e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Plan" sheetId="8" r:id="R58677b5b5fa74174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="9" r:id="Rfd03dbf4708d45ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R8ad5995011ce416d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test case List" sheetId="2" r:id="R2cd72f1e78904743"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestDesign" sheetId="3" r:id="R854b889adf6c4999"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_EMP" sheetId="4" r:id="Raafaa8d228bf4a6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_PERSONAL" sheetId="5" r:id="R38d37f2bd46f4e52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_JOB" sheetId="6" r:id="Rfffd753b6b794fdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data" sheetId="7" r:id="R3db59ede649e410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Plan" sheetId="8" r:id="R1a600b6077ce4a87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="9" r:id="Rfc099f8e00ab4016"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -752,7 +752,7 @@
         <x:v>Automation tool</x:v>
       </x:c>
       <x:c r="C19" s="3" t="str">
-        <x:v>Katalon Recorder</x:v>
+        <x:v>Katalon Recorder (phần PIM của Võ Minh Nhựt)</x:v>
       </x:c>
       <x:c r="D19" s="3"/>
       <x:c r="E19" s="3"/>
@@ -5209,7 +5209,7 @@
         <x:v>Review và Git</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
-        <x:v>Review 75 TC; commit workbook trên nhánh nhat/asm6-pim. Tạo PR vào dev, xử lý góp ý rồi merge.</x:v>
+        <x:v>Review 75 TC; commit workbook trên nhánh nhut. Tạo PR vào dev, xử lý góp ý rồi merge.</x:v>
       </x:c>
       <x:c r="D14" s="3" t="str">
         <x:v>Workbook đúng tên; ảnh bằng chứng push/merge thật; nhóm trưởng tổng hợp sau review.</x:v>
@@ -5237,9 +5237,9 @@
       <x:c r="E16" s="3"/>
       <x:c r="F16" s="3"/>
     </x:row>
-    <x:row r="17" ht="38" customHeight="1">
+    <x:row r="17" ht="44" customHeight="1">
       <x:c r="A17" s="3" t="str">
-        <x:v>P1/P2 là thứ tự ưu tiên triển khai, không phải kết quả chạy. Workbook hiện là test design; automation scripts chưa được triển khai.</x:v>
+        <x:v>Katalon Recorder là lựa chọn cá nhân của Võ Minh Nhựt. Các thành viên tự chọn công cụ. P1/P2 là mức ưu tiên triển khai, không phải kết quả chạy. Chưa triển khai automation scripts.</x:v>
       </x:c>
       <x:c r="B17" s="3"/>
       <x:c r="C17" s="3"/>

</xml_diff>

<commit_message>
feat: complete Personal Details and Job automation with verified results
</commit_message>
<xml_diff>
--- a/docs/test-cases/members/Group01_23130226_VoMinhNhut.xlsx
+++ b/docs/test-cases/members/Group01_23130226_VoMinhNhut.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R6ce442db74254706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test case List" sheetId="2" r:id="Rcf3bc50c930e48c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestDesign" sheetId="3" r:id="R5244d612e7a94695"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_EMP" sheetId="4" r:id="Rf177865332a54550"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_PERSONAL" sheetId="5" r:id="Rdf5d619283984c5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_JOB" sheetId="6" r:id="R387e8a31527649b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data" sheetId="7" r:id="R1b3dea0b060f41ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Plan" sheetId="8" r:id="R623cd4ee93ef4295"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="9" r:id="R53df4e1004b046f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R6d0d11ae6bbf48a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test case List" sheetId="2" r:id="Rb41220be63b54171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestDesign" sheetId="3" r:id="R6532fe6029fa4c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_EMP" sheetId="4" r:id="R65dd86b030be458d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_PERSONAL" sheetId="5" r:id="Rc83fd22ed7d84e85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIM_JOB" sheetId="6" r:id="R229fe1a914024d89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data" sheetId="7" r:id="R9fbcc5d7e76244eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Plan" sheetId="8" r:id="R4919aa0f294747b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="9" r:id="R995e104dded1496a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -543,11 +543,6 @@
     <x:t xml:space="preserve">Không phụ thuộc TC khác; dùng fixture setup.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_01
-Positive; Phân vùng tương đương
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">First Name bắt buộc</x:t>
   </x:si>
   <x:si>
@@ -562,11 +557,6 @@
     <x:t xml:space="preserve">First Name hiển thị Required. Không lưu tên rỗng; giá trị cũ còn nguyên sau tải lại.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_02
-Negative; Phân vùng tương đương
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Last Name bắt buộc</x:t>
   </x:si>
   <x:si>
@@ -595,11 +585,6 @@
     <x:t xml:space="preserve">Lưu nguyên 30 ký tự và không có lỗi giới hạn.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_02
-Positive; Phân tích giá trị biên
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">First Name vượt giới hạn 30 ký tự</x:t>
   </x:si>
   <x:si>
@@ -614,11 +599,6 @@
     <x:t xml:space="preserve">Có lỗi giới hạn 30 ký tự; không lưu chuỗi vượt giới hạn. Nếu UI chặn nhập, ghi rõ giới hạn thực tế.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_02
-Negative; Phân tích giá trị biên
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Middle Name vượt giới hạn 30 ký tự</x:t>
   </x:si>
   <x:si>
@@ -655,11 +635,6 @@
     <x:t xml:space="preserve">ID mới 10 ký tự được lưu nguyên và hồ sơ vẫn là F_PERSON.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_03
-Positive; Phân tích giá trị biên
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Employee Id dài 11 ký tự</x:t>
   </x:si>
   <x:si>
@@ -674,11 +649,6 @@
     <x:t xml:space="preserve">Có lỗi giới hạn 10 ký tự, không lưu ID 11 ký tự.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_03
-Negative; Phân tích giá trị biên
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Other Id dài 30 ký tự</x:t>
   </x:si>
   <x:si>
@@ -743,11 +713,6 @@
     <x:t xml:space="preserve">Lưu đúng ngày 29/02/2000. Không có lỗi định dạng ngày.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_04
-Positive; Phân vùng tương đương
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Date of Birth là ngày không tồn tại</x:t>
   </x:si>
   <x:si>
@@ -762,11 +727,6 @@
     <x:t xml:space="preserve">Hiển thị lỗi ngày/định dạng; không lưu ngày 30/02/2000.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_04
-Negative; Phân vùng tương đương
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">License Expiry Date hợp lệ</x:t>
   </x:si>
   <x:si>
@@ -851,11 +811,6 @@
     <x:t xml:space="preserve">Có đúng một dòng tệp mới với tên và mô tả đã nhập. Tệp tải về đọc được.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_05
-Positive; Chuyển trạng thái
-Automation: P2</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Không chọn file khi thêm attachment</x:t>
   </x:si>
   <x:si>
@@ -870,11 +825,6 @@
     <x:t xml:space="preserve">Trường file hiển thị Required. Không xuất hiện dòng attachment mới.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_05
-Negative; Phân vùng tương đương
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Mô tả attachment đúng 200 ký tự</x:t>
   </x:si>
   <x:si>
@@ -889,11 +839,6 @@
     <x:t xml:space="preserve">Attachment được lưu. Mô tả có đủ 200 ký tự, không bị cắt.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_05
-Positive; Phân tích giá trị biên
-Automation: P2</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Mô tả attachment vượt 200 ký tự</x:t>
   </x:si>
   <x:si>
@@ -908,11 +853,6 @@
     <x:t xml:space="preserve">Có lỗi giới hạn 200 ký tự. Không lưu mô tả vượt giới hạn.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_05
-Negative; Phân tích giá trị biên
-Automation: P2</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Hủy rồi xác nhận xóa attachment của nhóm</x:t>
   </x:si>
   <x:si>
@@ -927,12 +867,6 @@
     <x:t xml:space="preserve">Sau Cancel, tệp vẫn có. Sau xác nhận xóa, đúng tệp đích biến mất và các tệp khác không thay đổi.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_PERSONAL_05
-Integration; Chuyển trạng thái
-Automation: P2
-Chỉ xóa tệp fixture của nhóm.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Lưu Joined Date hợp lệ</x:t>
   </x:si>
   <x:si>
@@ -947,11 +881,6 @@
     <x:t xml:space="preserve">Joined Date được lưu đúng ngày 01/10/2024.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_01
-Positive; Phân vùng tương đương
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Joined Date không tồn tại</x:t>
   </x:si>
   <x:si>
@@ -966,11 +895,6 @@
     <x:t xml:space="preserve">Có lỗi ngày/định dạng. Không lưu ngày 31/02/2024.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_01
-Negative; Phân vùng tương đương
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Thay đổi Job Title</x:t>
   </x:si>
   <x:si>
@@ -985,11 +909,6 @@
     <x:t xml:space="preserve">Job Title giữ đúng nhãn đã chọn sau tải lại; không thay đổi nhân viên khác.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_02
-Positive; Phân vùng tương đương
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Thay đổi Job Category</x:t>
   </x:si>
   <x:si>
@@ -1060,11 +979,6 @@
     <x:t xml:space="preserve">Ngày và toàn bộ 5 danh mục đều giữ đúng giá trị đã lưu trên F_JOB.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_02
-Integration; Bảng quyết định
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Xóa Joined Date tùy chọn</x:t>
   </x:si>
   <x:si>
@@ -1093,11 +1007,6 @@
     <x:t xml:space="preserve">Hiển thị Start Date, End Date và vùng Contract Details/upload. Không coi thao tác bật là bằng chứng đã lưu hợp đồng.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_03
-Positive; Phân vùng tương đương
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Tắt phần mở rộng hợp đồng không xóa dữ liệu</x:t>
   </x:si>
   <x:si>
@@ -1112,11 +1021,6 @@
     <x:t xml:space="preserve">Phần hợp đồng ẩn rồi hiện. Ngày và tệp vẫn còn khi bật lại. Không tự xóa dữ liệu do thao tác toggle.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_03
-Positive; Chuyển trạng thái
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Hợp đồng có End Date sau Start Date</x:t>
   </x:si>
   <x:si>
@@ -1131,11 +1035,6 @@
     <x:t xml:space="preserve">Lưu đúng hai ngày. End Date sau Start Date, không có lỗi.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_04
-Positive; Bảng quyết định
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">End Date trước Start Date</x:t>
   </x:si>
   <x:si>
@@ -1150,11 +1049,6 @@
     <x:t xml:space="preserve">End Date có lỗi yêu cầu sau Start Date. Không lưu cặp ngày sai.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_04
-Negative; Bảng quyết định
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">End Date bằng Start Date</x:t>
   </x:si>
   <x:si>
@@ -1169,11 +1063,6 @@
     <x:t xml:space="preserve">End Date bị từ chối vì phải sau Start Date (không chấp nhận cùng ngày theo baseline 5.9).</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_04
-Negative; Phân tích giá trị biên
-Automation: P1</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Start Date không tồn tại</x:t>
   </x:si>
   <x:si>
@@ -1185,11 +1074,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Có lỗi ngày/định dạng tại Start Date. Không lưu ngày không tồn tại.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_04
-Negative; Phân vùng tương đương
-Automation: P1</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">End Date không tồn tại</x:t>
@@ -1219,11 +1103,6 @@
     <x:t xml:space="preserve">Tên contract_v1.pdf còn sau tải lại. Nội dung tải xuống là hợp đồng mẫu v1.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_05
-Positive; Chuyển trạng thái
-Automation: P2</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Từ chối tệp hợp đồng vượt giới hạn</x:t>
   </x:si>
   <x:si>
@@ -1238,12 +1117,6 @@
     <x:t xml:space="preserve">Có lỗi dung lượng. Tệp hợp đồng cũ không bị thay bằng tệp quá cỡ.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_05
-Negative; Phân tích giá trị biên
-Automation: P2
-Không mặc định giới hạn contract giống ảnh đại diện.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Từ chối loại file hợp đồng không cho phép</x:t>
   </x:si>
   <x:si>
@@ -1258,11 +1131,6 @@
     <x:t xml:space="preserve">Có lỗi loại tệp. Không lưu tệp không được phép, hợp đồng cũ còn nguyên.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_05
-Negative; Phân vùng tương đương
-Automation: P2</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Giữ tệp hợp đồng hiện tại khi đổi ngày</x:t>
   </x:si>
   <x:si>
@@ -1277,11 +1145,6 @@
     <x:t xml:space="preserve">Ngày kết thúc mới được lưu. Tệp vẫn là contract_v1.pdf, nội dung không đổi.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_05
-Integration; Chuyển trạng thái
-Automation: P2</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Thay thế tệp hợp đồng hiện tại</x:t>
   </x:si>
   <x:si>
@@ -1310,11 +1173,6 @@
     <x:t xml:space="preserve">Vùng tệp mới hiển thị Required. Không mất tệp hợp đồng cũ.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_05
-Negative; Bảng quyết định
-Automation: P2</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Xóa riêng tệp hợp đồng hiện tại</x:t>
   </x:si>
   <x:si>
@@ -1329,12 +1187,6 @@
     <x:t xml:space="preserve">Tệp hiện tại được xóa. Hai ngày hợp đồng không bị đổi ngoài ý muốn.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_05
-Positive; Chuyển trạng thái
-Automation: P2
-Chỉ xóa tệp fixture của nhóm.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Thêm attachment tại tab Job</x:t>
   </x:si>
   <x:si>
@@ -1363,11 +1215,6 @@
     <x:t xml:space="preserve">Form thêm đóng. Không có dòng mới với mô tả G01N01 Job cancel.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TD_PIM_JOB_05
-Negative; Chuyển trạng thái
-Automation: P2</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">PIM TEST DATA</x:t>
   </x:si>
   <x:si>
@@ -1638,16 +1485,7 @@
     <x:t xml:space="preserve">ATTACH_LIMIT</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Giá trị hiện tại: điền trước run</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Đọc Max Attachment Size và Allowed File Types tại cấu hình hoặc hint. Ghi giới hạn, MIME và thời điểm.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Tệp quá giới hạn = giới hạn byte +1. Không đổi config dùng chung.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Nếu không đọc được config thì Blocked, không phỏng đoán.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">RESTORE</x:t>
@@ -2604,7 +2442,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="G7" s="35" t="str">
-        <x:v>1.2</x:v>
+        <x:v>1.3</x:v>
       </x:c>
       <x:c r="H7" s="2"/>
     </x:row>
@@ -2776,7 +2614,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C19" s="35" t="str">
-        <x:v>Playwright (PIM_EMP); các thành viên tự chọn công cụ</x:v>
+        <x:v>Playwright</x:v>
       </x:c>
       <x:c r="D19" s="39"/>
       <x:c r="E19" s="39"/>
@@ -2811,7 +2649,7 @@
         <x:v>Nội dung tuần này</x:v>
       </x:c>
       <x:c r="C22" t="str">
-        <x:v>PIM_EMP: Employee List &amp; Add Employee – 25 test case.</x:v>
+        <x:v>Thực thi PIM_PERSONAL và PIM_JOB: 50 test case.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1"/>
@@ -8605,7 +8443,7 @@
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="41" t="n">
         <x:f>COUNTIF($F$9:$F$33,"Passed")</x:f>
-        <x:v>0</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF($F$9:$F$33,"Failed")</x:f>
@@ -8613,7 +8451,7 @@
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF($F$9:$F$33,"Untested")</x:f>
-        <x:v>25</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="41" t="n">
         <x:f>COUNTIF($F$9:$F$33,"Blocked")</x:f>
@@ -8666,7 +8504,7 @@
         <x:v>60</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="139.5" customHeight="1">
+    <x:row r="9" ht="210" customHeight="1">
       <x:c r="A9" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_01</x:v>
       </x:c>
@@ -8682,588 +8520,848 @@
       <x:c r="E9" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F9" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G9" s="44"/>
-      <x:c r="H9" s="42" t="s">
-        <x:v>169</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="139.5" customHeight="1">
+      <x:c r="F9" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G9" s="44" t="d">
+        <x:v>2026-10-28T03:07:03.617Z</x:v>
+      </x:c>
+      <x:c r="H9" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_01
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Cập nhật đầy đủ ba thành phần tên
+Time: 6.36s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="210" customHeight="1">
       <x:c r="A10" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_02</x:v>
       </x:c>
       <x:c r="B10" s="45" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="C10" s="45" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="C10" s="45" t="s">
+      <x:c r="D10" s="45" t="s">
         <x:v>171</x:v>
-      </x:c>
-      <x:c r="D10" s="45" t="s">
-        <x:v>172</x:v>
       </x:c>
       <x:c r="E10" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F10" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G10" s="44"/>
-      <x:c r="H10" s="42" t="s">
-        <x:v>173</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="139.5" customHeight="1">
+      <x:c r="F10" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G10" s="44" t="d">
+        <x:v>2026-10-28T03:07:08.549Z</x:v>
+      </x:c>
+      <x:c r="H10" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_02
+Negative; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: First Name bắt buộc | Required | Saved value unchanged after reopening
+Time: 4.93s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_02-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="210" customHeight="1">
       <x:c r="A11" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_03</x:v>
       </x:c>
       <x:c r="B11" s="42" t="s">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="C11" s="42" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D11" s="42" t="s">
         <x:v>174</x:v>
-      </x:c>
-      <x:c r="C11" s="42" t="s">
-        <x:v>175</x:v>
-      </x:c>
-      <x:c r="D11" s="42" t="s">
-        <x:v>176</x:v>
       </x:c>
       <x:c r="E11" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F11" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G11" s="44"/>
-      <x:c r="H11" s="42" t="s">
-        <x:v>173</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="139.5" customHeight="1">
+      <x:c r="F11" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G11" s="44" t="d">
+        <x:v>2026-10-28T03:07:13.578Z</x:v>
+      </x:c>
+      <x:c r="H11" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_02
+Negative; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Last Name bắt buộc | Required | Saved value unchanged after reopening
+Time: 5.03s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_03-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="233" customHeight="1">
       <x:c r="A12" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_04</x:v>
       </x:c>
       <x:c r="B12" s="45" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="C12" s="45" t="s">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="D12" s="45" t="s">
         <x:v>177</x:v>
-      </x:c>
-      <x:c r="C12" s="45" t="s">
-        <x:v>178</x:v>
-      </x:c>
-      <x:c r="D12" s="45" t="s">
-        <x:v>179</x:v>
       </x:c>
       <x:c r="E12" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F12" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G12" s="44"/>
-      <x:c r="H12" s="42" t="s">
-        <x:v>180</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="139.5" customHeight="1">
+      <x:c r="F12" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G12" s="44" t="d">
+        <x:v>2026-10-28T03:07:19.477Z</x:v>
+      </x:c>
+      <x:c r="H12" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_02
+Positive; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: First Name đúng giới hạn 30 ký tự
+Input:
+value: AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA
+Time: 5.90s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_04-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="259" customHeight="1">
       <x:c r="A13" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_05</x:v>
       </x:c>
       <x:c r="B13" s="42" t="s">
-        <x:v>181</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C13" s="42" t="s">
-        <x:v>182</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="D13" s="42" t="s">
-        <x:v>183</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="E13" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F13" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G13" s="44"/>
-      <x:c r="H13" s="42" t="s">
-        <x:v>184</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="139.5" customHeight="1">
+      <x:c r="F13" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G13" s="44" t="d">
+        <x:v>2026-10-28T03:07:24.518Z</x:v>
+      </x:c>
+      <x:c r="H13" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_02
+Negative; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: First Name vượt giới hạn 30 ký tự | Should not exceed 30 characters | Saved value unchanged after reopening
+Input:
+value: AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA
+Time: 5.04s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_05-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="259" customHeight="1">
       <x:c r="A14" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_06</x:v>
       </x:c>
       <x:c r="B14" s="45" t="s">
-        <x:v>185</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C14" s="45" t="s">
-        <x:v>186</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="D14" s="45" t="s">
-        <x:v>183</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="E14" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F14" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G14" s="44"/>
-      <x:c r="H14" s="42" t="s">
-        <x:v>184</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="139.5" customHeight="1">
+      <x:c r="F14" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G14" s="44" t="d">
+        <x:v>2026-10-28T03:07:29.794Z</x:v>
+      </x:c>
+      <x:c r="H14" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_02
+Negative; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Middle Name vượt giới hạn 30 ký tự | Should not exceed 30 characters | Saved value unchanged after reopening
+Input:
+value: AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA
+Time: 5.27s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_06-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="259" customHeight="1">
       <x:c r="A15" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_07</x:v>
       </x:c>
       <x:c r="B15" s="42" t="s">
-        <x:v>187</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="C15" s="42" t="s">
-        <x:v>188</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="D15" s="42" t="s">
-        <x:v>183</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="E15" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F15" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G15" s="44"/>
-      <x:c r="H15" s="42" t="s">
-        <x:v>184</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="139.5" customHeight="1">
+      <x:c r="F15" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G15" s="44" t="d">
+        <x:v>2026-10-28T03:07:34.794Z</x:v>
+      </x:c>
+      <x:c r="H15" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_02
+Negative; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Last Name vượt giới hạn 30 ký tự | Should not exceed 30 characters | Saved value unchanged after reopening
+Input:
+value: AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA
+Time: 5.00s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_07-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="210" customHeight="1">
       <x:c r="A16" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_08</x:v>
       </x:c>
       <x:c r="B16" s="45" t="s">
-        <x:v>189</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="C16" s="45" t="s">
-        <x:v>190</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="D16" s="45" t="s">
-        <x:v>191</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="E16" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F16" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G16" s="44"/>
-      <x:c r="H16" s="42" t="s">
-        <x:v>192</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="139.5" customHeight="1">
+      <x:c r="F16" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G16" s="44" t="d">
+        <x:v>2026-10-28T03:07:49.309Z</x:v>
+      </x:c>
+      <x:c r="H16" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_03
+Positive; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Employee Id dài 10 ký tự
+Input:
+value: T2536ee39b
+Time: 14.51s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_08-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="246" customHeight="1">
       <x:c r="A17" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_09</x:v>
       </x:c>
       <x:c r="B17" s="42" t="s">
-        <x:v>193</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="C17" s="42" t="s">
-        <x:v>194</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="D17" s="42" t="s">
-        <x:v>195</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="E17" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F17" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G17" s="44"/>
-      <x:c r="H17" s="42" t="s">
-        <x:v>196</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="139.5" customHeight="1">
+      <x:c r="F17" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G17" s="44" t="d">
+        <x:v>2026-10-28T03:07:54.319Z</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_03
+Negative; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Employee Id dài 11 ký tự | Should not exceed 10 characters | Saved value unchanged after reopening
+Input:
+value: T2536ee39bX
+Time: 5.01s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_09-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="220" customHeight="1">
       <x:c r="A18" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_10</x:v>
       </x:c>
       <x:c r="B18" s="45" t="s">
-        <x:v>197</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C18" s="45" t="s">
-        <x:v>198</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D18" s="45" t="s">
-        <x:v>199</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="E18" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F18" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G18" s="44"/>
-      <x:c r="H18" s="42" t="s">
-        <x:v>192</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="139.5" customHeight="1">
+      <x:c r="F18" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G18" s="44" t="d">
+        <x:v>2026-10-28T03:08:00.257Z</x:v>
+      </x:c>
+      <x:c r="H18" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_03
+Positive; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Other Id dài 30 ký tự
+Input:
+value: BBBBBBBBBBBBBBBBBBBBBBBBBBBBBB
+Time: 5.94s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_10-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="246" customHeight="1">
       <x:c r="A19" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_11</x:v>
       </x:c>
       <x:c r="B19" s="42" t="s">
-        <x:v>200</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C19" s="42" t="s">
-        <x:v>201</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D19" s="42" t="s">
-        <x:v>202</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="E19" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F19" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G19" s="44"/>
-      <x:c r="H19" s="42" t="s">
-        <x:v>196</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="139.5" customHeight="1">
+      <x:c r="F19" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G19" s="44" t="d">
+        <x:v>2026-10-28T03:08:05.310Z</x:v>
+      </x:c>
+      <x:c r="H19" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_03
+Negative; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Other Id dài 31 ký tự | Should not exceed 30 characters | Saved value unchanged after reopening
+Input:
+value: BBBBBBBBBBBBBBBBBBBBBBBBBBBBBBB
+Time: 5.05s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_11-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="233" customHeight="1">
       <x:c r="A20" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_12</x:v>
       </x:c>
       <x:c r="B20" s="45" t="s">
-        <x:v>203</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="C20" s="45" t="s">
-        <x:v>204</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="D20" s="45" t="s">
-        <x:v>199</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="E20" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F20" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G20" s="44"/>
-      <x:c r="H20" s="42" t="s">
-        <x:v>192</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="139.5" customHeight="1">
+      <x:c r="F20" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G20" s="44" t="d">
+        <x:v>2026-10-28T03:08:11.187Z</x:v>
+      </x:c>
+      <x:c r="H20" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_03
+Positive; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Driver's License Number dài 30 ký tự
+Input:
+value: BBBBBBBBBBBBBBBBBBBBBBBBBBBBBB
+Time: 5.88s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_12-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="259" customHeight="1">
       <x:c r="A21" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_13</x:v>
       </x:c>
       <x:c r="B21" s="42" t="s">
-        <x:v>205</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="C21" s="42" t="s">
-        <x:v>206</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="D21" s="42" t="s">
-        <x:v>202</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="E21" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F21" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G21" s="44"/>
-      <x:c r="H21" s="42" t="s">
-        <x:v>196</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="139.5" customHeight="1">
+      <x:c r="F21" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G21" s="44" t="d">
+        <x:v>2026-10-28T03:08:16.163Z</x:v>
+      </x:c>
+      <x:c r="H21" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_03
+Negative; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Driver's License Number dài 31 ký tự | Should not exceed 30 characters | Saved value unchanged after reopening
+Input:
+value: BBBBBBBBBBBBBBBBBBBBBBBBBBBBBBB
+Time: 4.97s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_13-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="220" customHeight="1">
       <x:c r="A22" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_14</x:v>
       </x:c>
       <x:c r="B22" s="45" t="s">
-        <x:v>207</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="C22" s="45" t="s">
-        <x:v>208</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="D22" s="45" t="s">
-        <x:v>209</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="E22" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F22" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G22" s="44"/>
-      <x:c r="H22" s="42" t="s">
-        <x:v>210</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="139.5" customHeight="1">
+      <x:c r="F22" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G22" s="44" t="d">
+        <x:v>2026-10-28T03:08:21.974Z</x:v>
+      </x:c>
+      <x:c r="H22" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_04
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Date of Birth là ngày nhuận hợp lệ
+Input:
+Date of Birth: 2000-29-02
+Time: 5.81s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_14-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="246" customHeight="1">
       <x:c r="A23" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_15</x:v>
       </x:c>
       <x:c r="B23" s="42" t="s">
-        <x:v>211</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="C23" s="42" t="s">
-        <x:v>212</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="D23" s="42" t="s">
-        <x:v>213</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="E23" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F23" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G23" s="44"/>
-      <x:c r="H23" s="42" t="s">
-        <x:v>214</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="139.5" customHeight="1">
+      <x:c r="F23" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G23" s="44" t="d">
+        <x:v>2026-10-28T03:08:29.477Z</x:v>
+      </x:c>
+      <x:c r="H23" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_04
+Negative; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Date of Birth là ngày không tồn tại | Should be a valid date in yyyy-dd-mm format | Saved value unchanged after reopening
+Input:
+Date of Birth: 2000-30-02
+Time: 7.50s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_15-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="210" customHeight="1">
       <x:c r="A24" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_16</x:v>
       </x:c>
       <x:c r="B24" s="45" t="s">
-        <x:v>215</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="C24" s="45" t="s">
-        <x:v>216</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="D24" s="45" t="s">
-        <x:v>217</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="E24" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F24" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G24" s="44"/>
-      <x:c r="H24" s="42" t="s">
-        <x:v>210</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="139.5" customHeight="1">
+      <x:c r="F24" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G24" s="44" t="d">
+        <x:v>2026-10-28T03:08:41.006Z</x:v>
+      </x:c>
+      <x:c r="H24" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_04
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: License Expiry Date hợp lệ
+Input:
+License Expiry Date: 2030-31-12
+Time: 11.53s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_16-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="246" customHeight="1">
       <x:c r="A25" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_17</x:v>
       </x:c>
       <x:c r="B25" s="42" t="s">
-        <x:v>218</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="C25" s="42" t="s">
-        <x:v>219</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="D25" s="42" t="s">
-        <x:v>220</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="E25" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F25" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G25" s="44"/>
-      <x:c r="H25" s="42" t="s">
-        <x:v>214</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="139.5" customHeight="1">
+      <x:c r="F25" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G25" s="44" t="d">
+        <x:v>2026-10-28T03:08:56.398Z</x:v>
+      </x:c>
+      <x:c r="H25" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_04
+Negative; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: License Expiry Date không hợp lệ | Should be a valid date in yyyy-dd-mm format | Saved value unchanged after reopening
+Input:
+License Expiry Date: 2030-31-04
+Time: 15.39s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_17-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="210" customHeight="1">
       <x:c r="A26" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_18</x:v>
       </x:c>
       <x:c r="B26" s="45" t="s">
-        <x:v>221</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="C26" s="45" t="s">
-        <x:v>222</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="D26" s="45" t="s">
-        <x:v>223</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="E26" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F26" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G26" s="44"/>
-      <x:c r="H26" s="42" t="s">
-        <x:v>169</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="139.5" customHeight="1">
+      <x:c r="F26" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G26" s="44" t="d">
+        <x:v>2026-10-28T03:09:12.002Z</x:v>
+      </x:c>
+      <x:c r="H26" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_01
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Thay đổi Nationality
+Input:
+Nationality: Afghan
+Time: 15.60s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_18-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="210" customHeight="1">
       <x:c r="A27" s="42" t="str">
         <x:v>PIM_PERSONAL_Update_19</x:v>
       </x:c>
       <x:c r="B27" s="42" t="s">
-        <x:v>224</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="C27" s="42" t="s">
-        <x:v>225</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="D27" s="42" t="s">
-        <x:v>226</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="E27" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F27" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G27" s="44"/>
-      <x:c r="H27" s="42" t="s">
-        <x:v>169</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="139.5" customHeight="1">
+      <x:c r="F27" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G27" s="44" t="d">
+        <x:v>2026-10-28T03:09:19.261Z</x:v>
+      </x:c>
+      <x:c r="H27" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_01
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Thay đổi Marital Status
+Input:
+Marital Status: Married
+Time: 7.26s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_19-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="210" customHeight="1">
       <x:c r="A28" s="45" t="str">
         <x:v>PIM_PERSONAL_Update_20</x:v>
       </x:c>
       <x:c r="B28" s="45" t="s">
-        <x:v>227</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="C28" s="45" t="s">
-        <x:v>228</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="D28" s="45" t="s">
-        <x:v>229</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="E28" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F28" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G28" s="44"/>
-      <x:c r="H28" s="42" t="s">
-        <x:v>169</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="139.5" customHeight="1">
+      <x:c r="F28" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G28" s="44" t="d">
+        <x:v>2026-10-28T03:09:25.120Z</x:v>
+      </x:c>
+      <x:c r="H28" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_01
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Thay đổi Gender
+Input:
+Gender: Female
+Time: 5.86s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_Update_20-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="210" customHeight="1">
       <x:c r="A29" s="42" t="str">
         <x:v>PIM_PERSONAL_CreateAttachment_01</x:v>
       </x:c>
       <x:c r="B29" s="42" t="s">
-        <x:v>230</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="C29" s="42" t="s">
-        <x:v>231</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="D29" s="42" t="s">
-        <x:v>232</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="E29" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F29" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G29" s="44"/>
-      <x:c r="H29" s="42" t="s">
-        <x:v>233</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="139.5" customHeight="1">
+      <x:c r="F29" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G29" s="44" t="d">
+        <x:v>2026-10-28T03:09:34.459Z</x:v>
+      </x:c>
+      <x:c r="H29" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_05
+Positive; Chuyển trạng thái
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Thêm attachment hợp lệ vào Personal Details
+Time: 9.34s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_CreateAttachment_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="210" customHeight="1">
       <x:c r="A30" s="45" t="str">
         <x:v>PIM_PERSONAL_CreateAttachment_02</x:v>
       </x:c>
       <x:c r="B30" s="45" t="s">
-        <x:v>234</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="C30" s="45" t="s">
-        <x:v>235</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="D30" s="45" t="s">
-        <x:v>236</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="E30" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F30" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G30" s="44"/>
-      <x:c r="H30" s="42" t="s">
-        <x:v>237</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="156" customHeight="1">
+      <x:c r="F30" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G30" s="44" t="d">
+        <x:v>2026-10-28T03:09:39.644Z</x:v>
+      </x:c>
+      <x:c r="H30" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_05
+Negative; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Không chọn file khi thêm attachment
+Time: 5.18s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_CreateAttachment_02-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="210" customHeight="1">
       <x:c r="A31" s="42" t="str">
         <x:v>PIM_PERSONAL_CreateAttachment_03</x:v>
       </x:c>
       <x:c r="B31" s="42" t="s">
-        <x:v>238</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="C31" s="42" t="s">
-        <x:v>239</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="D31" s="42" t="s">
-        <x:v>240</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="E31" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F31" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G31" s="44"/>
-      <x:c r="H31" s="42" t="s">
-        <x:v>241</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="156" customHeight="1">
+      <x:c r="F31" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G31" s="44" t="d">
+        <x:v>2026-10-28T03:09:48.631Z</x:v>
+      </x:c>
+      <x:c r="H31" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_05
+Positive; Phân tích giá trị biên
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Mô tả attachment đúng 200 ký tự
+Time: 8.99s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_CreateAttachment_03-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="210" customHeight="1">
       <x:c r="A32" s="45" t="str">
         <x:v>PIM_PERSONAL_CreateAttachment_04</x:v>
       </x:c>
       <x:c r="B32" s="45" t="s">
-        <x:v>242</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="C32" s="45" t="s">
-        <x:v>243</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="D32" s="45" t="s">
-        <x:v>244</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="E32" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F32" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G32" s="44"/>
-      <x:c r="H32" s="42" t="s">
-        <x:v>245</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="139.5" customHeight="1">
+      <x:c r="F32" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G32" s="44" t="d">
+        <x:v>2026-10-28T03:09:53.738Z</x:v>
+      </x:c>
+      <x:c r="H32" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_05
+Negative; Phân tích giá trị biên
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Mô tả attachment vượt 200 ký tự
+Time: 5.11s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_CreateAttachment_04-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="210" customHeight="1">
       <x:c r="A33" s="42" t="str">
         <x:v>PIM_PERSONAL_DeleteAttachment_01</x:v>
       </x:c>
       <x:c r="B33" s="42" t="s">
-        <x:v>246</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="C33" s="42" t="s">
-        <x:v>247</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="D33" s="42" t="s">
-        <x:v>248</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="E33" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F33" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G33" s="44"/>
-      <x:c r="H33" s="42" t="s">
-        <x:v>249</x:v>
+      <x:c r="F33" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G33" s="44" t="d">
+        <x:v>2026-10-28T03:10:05.740Z</x:v>
+      </x:c>
+      <x:c r="H33" s="42" t="str">
+        <x:v>TD_PIM_PERSONAL_05
+Integration; Chuyển trạng thái
+Automation: P2
+Chỉ xóa tệp fixture của nhóm.
+Playwright / Edge 156.0.4314.50
+Actual: Hủy rồi xác nhận xóa attachment của nhóm
+Time: 12.00s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-06-34-596Z/screenshots/PIM_PERSONAL_DeleteAttachment_01-result.png</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15.75" customHeight="1"/>
@@ -10365,7 +10463,7 @@
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="41" t="n">
         <x:f>COUNTIF($F$9:$F$33,"Passed")</x:f>
-        <x:v>0</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF($F$9:$F$33,"Failed")</x:f>
@@ -10373,7 +10471,7 @@
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF($F$9:$F$33,"Untested")</x:f>
-        <x:v>25</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="41" t="n">
         <x:f>COUNTIF($F$9:$F$33,"Blocked")</x:f>
@@ -10426,604 +10524,874 @@
         <x:v>60</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="139.5" customHeight="1">
+    <x:row r="9" ht="210" customHeight="1">
       <x:c r="A9" s="42" t="str">
         <x:v>PIM_JOB_UpdateJob_01</x:v>
       </x:c>
       <x:c r="B9" s="42" t="s">
-        <x:v>250</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="C9" s="42" t="s">
-        <x:v>251</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="D9" s="42" t="s">
-        <x:v>252</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="E9" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F9" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G9" s="44"/>
-      <x:c r="H9" s="42" t="s">
-        <x:v>253</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="139.5" customHeight="1">
+      <x:c r="F9" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G9" s="44" t="d">
+        <x:v>2026-10-28T03:14:59.490Z</x:v>
+      </x:c>
+      <x:c r="H9" s="42" t="str">
+        <x:v>TD_PIM_JOB_01
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Lưu Joined Date hợp lệ
+Input:
+JoinedDate: 2024-01-10
+Time: 7.10s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateJob_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="246" customHeight="1">
       <x:c r="A10" s="45" t="str">
         <x:v>PIM_JOB_UpdateJob_02</x:v>
       </x:c>
       <x:c r="B10" s="45" t="s">
-        <x:v>254</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="C10" s="45" t="s">
-        <x:v>255</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="D10" s="45" t="s">
-        <x:v>256</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="E10" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F10" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G10" s="44"/>
-      <x:c r="H10" s="42" t="s">
-        <x:v>257</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="139.5" customHeight="1">
+      <x:c r="F10" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G10" s="44" t="d">
+        <x:v>2026-10-28T03:15:04.751Z</x:v>
+      </x:c>
+      <x:c r="H10" s="42" t="str">
+        <x:v>TD_PIM_JOB_01
+Negative; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Joined Date không tồn tại | Should be a valid date in yyyy-dd-mm format | Saved value unchanged after reopening
+Input:
+JoinedDate: 2024-31-02
+Time: 5.26s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateJob_02-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="210" customHeight="1">
       <x:c r="A11" s="42" t="str">
         <x:v>PIM_JOB_UpdateJob_03</x:v>
       </x:c>
       <x:c r="B11" s="42" t="s">
-        <x:v>258</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="C11" s="42" t="s">
-        <x:v>259</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="D11" s="42" t="s">
-        <x:v>260</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="E11" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F11" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G11" s="44"/>
-      <x:c r="H11" s="42" t="s">
-        <x:v>261</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="139.5" customHeight="1">
+      <x:c r="F11" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G11" s="44" t="d">
+        <x:v>2026-10-28T03:15:11.313Z</x:v>
+      </x:c>
+      <x:c r="H11" s="42" t="str">
+        <x:v>TD_PIM_JOB_02
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Thay đổi Job Title
+Input:
+Job Title: Account Assistant
+Time: 6.56s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateJob_03-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="210" customHeight="1">
       <x:c r="A12" s="45" t="str">
         <x:v>PIM_JOB_UpdateJob_04</x:v>
       </x:c>
       <x:c r="B12" s="45" t="s">
-        <x:v>262</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="C12" s="45" t="s">
-        <x:v>263</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="D12" s="45" t="s">
-        <x:v>264</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="E12" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F12" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G12" s="44"/>
-      <x:c r="H12" s="42" t="s">
-        <x:v>261</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="139.5" customHeight="1">
+      <x:c r="F12" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G12" s="44" t="d">
+        <x:v>2026-10-28T03:15:18.205Z</x:v>
+      </x:c>
+      <x:c r="H12" s="42" t="str">
+        <x:v>TD_PIM_JOB_02
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Thay đổi Job Category
+Input:
+Job Category: Craft Workers
+Time: 6.89s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateJob_04-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="210" customHeight="1">
       <x:c r="A13" s="42" t="str">
         <x:v>PIM_JOB_UpdateJob_05</x:v>
       </x:c>
       <x:c r="B13" s="42" t="s">
-        <x:v>265</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="C13" s="42" t="s">
-        <x:v>266</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="D13" s="42" t="s">
-        <x:v>267</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="E13" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F13" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G13" s="44"/>
-      <x:c r="H13" s="42" t="s">
-        <x:v>261</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="139.5" customHeight="1">
+      <x:c r="F13" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G13" s="44" t="d">
+        <x:v>2026-10-28T03:15:24.592Z</x:v>
+      </x:c>
+      <x:c r="H13" s="42" t="str">
+        <x:v>TD_PIM_JOB_02
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Thay đổi Sub Unit
+Input:
+Sub Unit: Administration
+Time: 6.39s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateJob_05-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="210" customHeight="1">
       <x:c r="A14" s="45" t="str">
         <x:v>PIM_JOB_UpdateJob_06</x:v>
       </x:c>
       <x:c r="B14" s="45" t="s">
-        <x:v>268</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="C14" s="45" t="s">
-        <x:v>269</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="D14" s="45" t="s">
-        <x:v>270</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="E14" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F14" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G14" s="44"/>
-      <x:c r="H14" s="42" t="s">
-        <x:v>261</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="139.5" customHeight="1">
+      <x:c r="F14" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G14" s="44" t="d">
+        <x:v>2026-10-28T03:15:31.153Z</x:v>
+      </x:c>
+      <x:c r="H14" s="42" t="str">
+        <x:v>TD_PIM_JOB_02
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Thay đổi Location
+Input:
+Location: Canadian Regional HQ
+Time: 6.56s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateJob_06-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="210" customHeight="1">
       <x:c r="A15" s="42" t="str">
         <x:v>PIM_JOB_UpdateJob_07</x:v>
       </x:c>
       <x:c r="B15" s="42" t="s">
-        <x:v>271</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="C15" s="42" t="s">
-        <x:v>272</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="D15" s="42" t="s">
-        <x:v>273</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="E15" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F15" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G15" s="44"/>
-      <x:c r="H15" s="42" t="s">
-        <x:v>261</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="139.5" customHeight="1">
+      <x:c r="F15" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G15" s="44" t="d">
+        <x:v>2026-10-28T03:15:37.764Z</x:v>
+      </x:c>
+      <x:c r="H15" s="42" t="str">
+        <x:v>TD_PIM_JOB_02
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Thay đổi Employment Status
+Input:
+Employment Status: Freelance
+Time: 6.61s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateJob_07-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="285" customHeight="1">
       <x:c r="A16" s="45" t="str">
         <x:v>PIM_JOB_UpdateJob_08</x:v>
       </x:c>
       <x:c r="B16" s="45" t="s">
-        <x:v>274</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="C16" s="45" t="s">
-        <x:v>275</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="D16" s="45" t="s">
-        <x:v>276</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="E16" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F16" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G16" s="44"/>
-      <x:c r="H16" s="42" t="s">
-        <x:v>277</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="139.5" customHeight="1">
+      <x:c r="F16" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G16" s="44" t="d">
+        <x:v>2026-10-28T03:15:47.340Z</x:v>
+      </x:c>
+      <x:c r="H16" s="42" t="str">
+        <x:v>TD_PIM_JOB_02
+Integration; Bảng quyết định
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Lưu đồng thời các trường Job Details
+Input:
+Job Title: Automaton Tester
+Job Category: Laborers and Helpers
+Sub Unit: Engineering
+Location: HQ - CA, USA
+Employment Status: Full-Time Contract
+Time: 9.57s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateJob_08-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="210" customHeight="1">
       <x:c r="A17" s="42" t="str">
         <x:v>PIM_JOB_UpdateJob_09</x:v>
       </x:c>
       <x:c r="B17" s="42" t="s">
-        <x:v>278</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="C17" s="42" t="s">
-        <x:v>279</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="D17" s="42" t="s">
-        <x:v>280</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="E17" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F17" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G17" s="44"/>
-      <x:c r="H17" s="42" t="s">
-        <x:v>253</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="139.5" customHeight="1">
+      <x:c r="F17" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G17" s="44" t="d">
+        <x:v>2026-10-28T03:15:58.927Z</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="str">
+        <x:v>TD_PIM_JOB_01
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Xóa Joined Date tùy chọn
+Input:
+JoinedDate: 
+Time: 11.59s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateJob_09-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="210" customHeight="1">
       <x:c r="A18" s="45" t="str">
         <x:v>PIM_JOB_ToggleContract_01</x:v>
       </x:c>
       <x:c r="B18" s="45" t="s">
-        <x:v>281</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="C18" s="45" t="s">
-        <x:v>282</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="D18" s="45" t="s">
-        <x:v>283</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="E18" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F18" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G18" s="44"/>
-      <x:c r="H18" s="42" t="s">
-        <x:v>284</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="139.5" customHeight="1">
+      <x:c r="F18" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G18" s="44" t="d">
+        <x:v>2026-10-28T03:16:02.811Z</x:v>
+      </x:c>
+      <x:c r="H18" s="42" t="str">
+        <x:v>TD_PIM_JOB_03
+Positive; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Bật hiển thị Employment Contract Details
+Time: 3.88s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_ToggleContract_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="210" customHeight="1">
       <x:c r="A19" s="42" t="str">
         <x:v>PIM_JOB_ToggleContract_02</x:v>
       </x:c>
       <x:c r="B19" s="42" t="s">
-        <x:v>285</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="C19" s="42" t="s">
-        <x:v>286</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="D19" s="42" t="s">
-        <x:v>287</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="E19" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F19" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G19" s="44"/>
-      <x:c r="H19" s="42" t="s">
-        <x:v>288</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="139.5" customHeight="1">
+      <x:c r="F19" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G19" s="44" t="d">
+        <x:v>2026-10-28T03:16:14.130Z</x:v>
+      </x:c>
+      <x:c r="H19" s="42" t="str">
+        <x:v>TD_PIM_JOB_03
+Positive; Chuyển trạng thái
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Tắt phần mở rộng hợp đồng không xóa dữ liệu
+Time: 11.32s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_ToggleContract_02-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="233" customHeight="1">
       <x:c r="A20" s="45" t="str">
         <x:v>PIM_JOB_UpdateContract_01</x:v>
       </x:c>
       <x:c r="B20" s="45" t="s">
-        <x:v>289</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="C20" s="45" t="s">
-        <x:v>290</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="D20" s="45" t="s">
-        <x:v>291</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="E20" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F20" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G20" s="44"/>
-      <x:c r="H20" s="42" t="s">
-        <x:v>292</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="139.5" customHeight="1">
+      <x:c r="F20" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G20" s="44" t="d">
+        <x:v>2026-10-28T03:16:22.733Z</x:v>
+      </x:c>
+      <x:c r="H20" s="42" t="str">
+        <x:v>TD_PIM_JOB_04
+Positive; Bảng quyết định
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Hợp đồng có End Date sau Start Date
+Input:
+start: 2026-01-01
+end: 2026-31-12
+Time: 8.60s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateContract_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="246" customHeight="1">
       <x:c r="A21" s="42" t="str">
         <x:v>PIM_JOB_UpdateContract_02</x:v>
       </x:c>
       <x:c r="B21" s="42" t="s">
-        <x:v>293</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="C21" s="42" t="s">
-        <x:v>294</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="D21" s="42" t="s">
-        <x:v>295</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="E21" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F21" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G21" s="44"/>
-      <x:c r="H21" s="42" t="s">
-        <x:v>296</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="139.5" customHeight="1">
+      <x:c r="F21" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G21" s="44" t="d">
+        <x:v>2026-10-28T03:16:30.004Z</x:v>
+      </x:c>
+      <x:c r="H21" s="42" t="str">
+        <x:v>TD_PIM_JOB_04
+Negative; Bảng quyết định
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: End Date trước Start Date | End date should be after Start date
+Input:
+start: 2026-01-01
+end: 2025-31-12
+Time: 7.27s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateContract_02-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="233" customHeight="1">
       <x:c r="A22" s="45" t="str">
         <x:v>PIM_JOB_UpdateContract_03</x:v>
       </x:c>
       <x:c r="B22" s="45" t="s">
-        <x:v>297</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="C22" s="45" t="s">
-        <x:v>298</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="D22" s="45" t="s">
-        <x:v>299</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="E22" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F22" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G22" s="44"/>
-      <x:c r="H22" s="42" t="s">
-        <x:v>300</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="139.5" customHeight="1">
+      <x:c r="F22" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G22" s="44" t="d">
+        <x:v>2026-10-28T03:16:37.258Z</x:v>
+      </x:c>
+      <x:c r="H22" s="42" t="str">
+        <x:v>TD_PIM_JOB_04
+Negative; Phân tích giá trị biên
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: End Date bằng Start Date | End date should be after Start date
+Input:
+start: 2026-01-01
+end: 2026-01-01
+Time: 7.25s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateContract_03-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="246" customHeight="1">
       <x:c r="A23" s="42" t="str">
         <x:v>PIM_JOB_UpdateContract_04</x:v>
       </x:c>
       <x:c r="B23" s="42" t="s">
-        <x:v>301</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="C23" s="42" t="s">
-        <x:v>302</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="D23" s="42" t="s">
-        <x:v>303</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="E23" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F23" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G23" s="44"/>
-      <x:c r="H23" s="42" t="s">
-        <x:v>304</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="139.5" customHeight="1">
+      <x:c r="F23" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G23" s="44" t="d">
+        <x:v>2026-10-28T03:16:44.973Z</x:v>
+      </x:c>
+      <x:c r="H23" s="42" t="str">
+        <x:v>TD_PIM_JOB_04
+Negative; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: Start Date không tồn tại | Should be a valid date in yyyy-dd-mm format
+Input:
+start: 2026-31-02
+end: 2026-31-12
+Time: 7.71s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateContract_04-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="246" customHeight="1">
       <x:c r="A24" s="45" t="str">
         <x:v>PIM_JOB_UpdateContract_05</x:v>
       </x:c>
       <x:c r="B24" s="45" t="s">
-        <x:v>305</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="C24" s="45" t="s">
-        <x:v>306</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D24" s="45" t="s">
-        <x:v>307</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="E24" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F24" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G24" s="44"/>
-      <x:c r="H24" s="42" t="s">
-        <x:v>304</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="139.5" customHeight="1">
+      <x:c r="F24" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G24" s="44" t="d">
+        <x:v>2026-10-28T03:16:52.462Z</x:v>
+      </x:c>
+      <x:c r="H24" s="42" t="str">
+        <x:v>TD_PIM_JOB_04
+Negative; Phân vùng tương đương
+Automation: P1
+Playwright / Edge 156.0.4314.50
+Actual: End Date không tồn tại | Should be a valid date in yyyy-dd-mm format
+Input:
+start: 2026-01-01
+end: 2026-31-04
+Time: 7.49s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UpdateContract_05-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="210" customHeight="1">
       <x:c r="A25" s="42" t="str">
         <x:v>PIM_JOB_UploadContract_01</x:v>
       </x:c>
       <x:c r="B25" s="42" t="s">
-        <x:v>308</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="C25" s="42" t="s">
-        <x:v>309</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="D25" s="42" t="s">
-        <x:v>310</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="E25" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F25" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G25" s="44"/>
-      <x:c r="H25" s="42" t="s">
-        <x:v>311</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="141.75" customHeight="1">
+      <x:c r="F25" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G25" s="44" t="d">
+        <x:v>2026-10-28T03:17:15.431Z</x:v>
+      </x:c>
+      <x:c r="H25" s="42" t="str">
+        <x:v>TD_PIM_JOB_05
+Positive; Chuyển trạng thái
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Tải tệp hợp đồng PDF hợp lệ
+Time: 22.97s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UploadContract_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="272" customHeight="1">
       <x:c r="A26" s="45" t="str">
         <x:v>PIM_JOB_UploadContract_02</x:v>
       </x:c>
       <x:c r="B26" s="45" t="s">
-        <x:v>312</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="C26" s="45" t="s">
-        <x:v>313</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="D26" s="45" t="s">
-        <x:v>314</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="E26" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F26" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G26" s="44"/>
-      <x:c r="H26" s="42" t="s">
-        <x:v>315</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="141.75" customHeight="1">
+      <x:c r="F26" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G26" s="44" t="d">
+        <x:v>2026-10-28T03:17:32.040Z</x:v>
+      </x:c>
+      <x:c r="H26" s="42" t="str">
+        <x:v>TD_PIM_JOB_05
+Negative; Phân tích giá trị biên
+Automation: P2
+Không mặc định giới hạn contract giống ảnh đại diện.
+Playwright / Edge 156.0.4314.50
+Actual: Từ chối tệp hợp đồng vượt giới hạn | Attachment Size Exceeded
+Input:
+hint: Accepts up to 1MB
+size: 1048577
+limit: 1048576
+Time: 16.61s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UploadContract_02-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="233" customHeight="1">
       <x:c r="A27" s="42" t="str">
         <x:v>PIM_JOB_UploadContract_03</x:v>
       </x:c>
       <x:c r="B27" s="42" t="s">
-        <x:v>316</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C27" s="42" t="s">
-        <x:v>317</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="D27" s="42" t="s">
-        <x:v>318</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E27" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F27" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G27" s="44"/>
-      <x:c r="H27" s="42" t="s">
-        <x:v>319</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="139.5" customHeight="1">
+      <x:c r="F27" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G27" s="44" t="d">
+        <x:v>2026-10-28T03:17:47.868Z</x:v>
+      </x:c>
+      <x:c r="H27" s="42" t="str">
+        <x:v>TD_PIM_JOB_05
+Negative; Phân vùng tương đương
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Từ chối loại file hợp đồng không cho phép | File type not allowed
+Input:
+filename: contract_disallowed.bin
+Time: 15.83s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_UploadContract_03-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="210" customHeight="1">
       <x:c r="A28" s="45" t="str">
         <x:v>PIM_JOB_KeepContract_01</x:v>
       </x:c>
       <x:c r="B28" s="45" t="s">
-        <x:v>320</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="C28" s="45" t="s">
-        <x:v>321</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="D28" s="45" t="s">
-        <x:v>322</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="E28" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F28" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G28" s="44"/>
-      <x:c r="H28" s="42" t="s">
-        <x:v>323</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="139.5" customHeight="1">
+      <x:c r="F28" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G28" s="44" t="d">
+        <x:v>2026-10-28T03:18:05.591Z</x:v>
+      </x:c>
+      <x:c r="H28" s="42" t="str">
+        <x:v>TD_PIM_JOB_05
+Integration; Chuyển trạng thái
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Giữ tệp hợp đồng hiện tại khi đổi ngày
+Time: 17.72s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_KeepContract_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="210" customHeight="1">
       <x:c r="A29" s="42" t="str">
         <x:v>PIM_JOB_ReplaceContract_01</x:v>
       </x:c>
       <x:c r="B29" s="42" t="s">
-        <x:v>324</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="C29" s="42" t="s">
-        <x:v>325</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="D29" s="42" t="s">
-        <x:v>326</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="E29" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F29" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G29" s="44"/>
-      <x:c r="H29" s="42" t="s">
-        <x:v>311</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="139.5" customHeight="1">
+      <x:c r="F29" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G29" s="44" t="d">
+        <x:v>2026-10-28T03:18:23.659Z</x:v>
+      </x:c>
+      <x:c r="H29" s="42" t="str">
+        <x:v>TD_PIM_JOB_05
+Positive; Chuyển trạng thái
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Thay thế tệp hợp đồng hiện tại
+Time: 18.07s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_ReplaceContract_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="210" customHeight="1">
       <x:c r="A30" s="45" t="str">
         <x:v>PIM_JOB_ReplaceContract_02</x:v>
       </x:c>
       <x:c r="B30" s="45" t="s">
-        <x:v>327</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C30" s="45" t="s">
-        <x:v>328</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="D30" s="45" t="s">
-        <x:v>329</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="E30" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F30" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G30" s="44"/>
-      <x:c r="H30" s="42" t="s">
-        <x:v>330</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="139.5" customHeight="1">
+      <x:c r="F30" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G30" s="44" t="d">
+        <x:v>2026-10-28T03:19:03.952Z</x:v>
+      </x:c>
+      <x:c r="H30" s="42" t="str">
+        <x:v>TD_PIM_JOB_05
+Negative; Bảng quyết định
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Replace Current nhưng không chọn tệp mới | Required
+Time: 40.29s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_ReplaceContract_02-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="210" customHeight="1">
       <x:c r="A31" s="42" t="str">
         <x:v>PIM_JOB_DeleteContract_01</x:v>
       </x:c>
       <x:c r="B31" s="42" t="s">
-        <x:v>331</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="C31" s="42" t="s">
-        <x:v>332</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="D31" s="42" t="s">
-        <x:v>333</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="E31" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F31" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G31" s="44"/>
-      <x:c r="H31" s="42" t="s">
-        <x:v>334</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="139.5" customHeight="1">
+      <x:c r="F31" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G31" s="44" t="d">
+        <x:v>2026-10-28T03:19:37.819Z</x:v>
+      </x:c>
+      <x:c r="H31" s="42" t="str">
+        <x:v>TD_PIM_JOB_05
+Positive; Chuyển trạng thái
+Automation: P2
+Chỉ xóa tệp fixture của nhóm.
+Playwright / Edge 156.0.4314.50
+Actual: Xóa riêng tệp hợp đồng hiện tại
+Time: 33.87s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_DeleteContract_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="210" customHeight="1">
       <x:c r="A32" s="45" t="str">
         <x:v>PIM_JOB_CreateAttachment_01</x:v>
       </x:c>
       <x:c r="B32" s="45" t="s">
-        <x:v>335</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="C32" s="45" t="s">
-        <x:v>336</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="D32" s="45" t="s">
-        <x:v>337</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="E32" s="45" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F32" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G32" s="44"/>
-      <x:c r="H32" s="42" t="s">
-        <x:v>311</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="139.5" customHeight="1">
+      <x:c r="F32" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G32" s="44" t="d">
+        <x:v>2026-10-28T03:19:54.952Z</x:v>
+      </x:c>
+      <x:c r="H32" s="42" t="str">
+        <x:v>TD_PIM_JOB_05
+Positive; Chuyển trạng thái
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Thêm attachment tại tab Job
+Time: 17.13s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_CreateAttachment_01-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="210" customHeight="1">
       <x:c r="A33" s="42" t="str">
         <x:v>PIM_JOB_CancelAttachment_01</x:v>
       </x:c>
       <x:c r="B33" s="42" t="s">
-        <x:v>338</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="C33" s="42" t="s">
-        <x:v>339</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="D33" s="42" t="s">
-        <x:v>340</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="E33" s="42" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F33" s="43" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G33" s="44"/>
-      <x:c r="H33" s="42" t="s">
-        <x:v>341</x:v>
+      <x:c r="F33" s="43" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G33" s="44" t="d">
+        <x:v>2026-10-28T03:20:01.794Z</x:v>
+      </x:c>
+      <x:c r="H33" s="42" t="str">
+        <x:v>TD_PIM_JOB_05
+Negative; Chuyển trạng thái
+Automation: P2
+Playwright / Edge 156.0.4314.50
+Actual: Hủy thêm attachment tại tab Job
+Time: 6.84s
+Log: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/results.json
+Ảnh: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/screenshots/PIM_JOB_CancelAttachment_01-result.png</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15.75" customHeight="1"/>
@@ -12053,7 +12421,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="3" t="s">
-        <x:v>342</x:v>
+        <x:v>312</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -12066,59 +12434,59 @@
     </x:row>
     <x:row r="4" ht="31.5" customHeight="1">
       <x:c r="A4" s="38" t="s">
-        <x:v>343</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="B4" s="38" t="s">
-        <x:v>344</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="C4" s="38" t="s">
-        <x:v>345</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="D4" s="38" t="s">
-        <x:v>346</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="E4" s="38" t="s">
-        <x:v>347</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="F4" s="38" t="s">
-        <x:v>348</x:v>
+        <x:v>318</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="109.5" customHeight="1">
       <x:c r="A5" s="35" t="s">
-        <x:v>349</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="B5" s="35" t="s">
-        <x:v>350</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C5" s="35" t="s">
-        <x:v>351</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D5" s="35" t="s">
-        <x:v>352</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="E5" s="35" t="s">
-        <x:v>353</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="F5" s="35" t="s">
-        <x:v>354</x:v>
+        <x:v>324</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="109.5" customHeight="1">
       <x:c r="A6" s="35" t="s">
-        <x:v>355</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="B6" s="35" t="s">
-        <x:v>356</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="C6" s="35" t="s">
-        <x:v>357</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="D6" s="35" t="s">
-        <x:v>358</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="E6" s="35" t="s">
-        <x:v>359</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="F6" s="35" t="str">
         <x:v>Tài khoản demo công khai; không thay mật khẩu.</x:v>
@@ -12126,230 +12494,230 @@
     </x:row>
     <x:row r="7" ht="109.5" customHeight="1">
       <x:c r="A7" s="35" t="s">
-        <x:v>360</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="B7" s="35" t="str">
         <x:v>ID=G1N01D0001; First=G01N01; Last=NhutDuplicate</x:v>
       </x:c>
       <x:c r="C7" s="35" t="s">
-        <x:v>361</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="D7" s="35" t="str">
         <x:v>PIM_EMP_Create_14; PIM_EMP_Search_01; PIM_EMP_Reset_01</x:v>
       </x:c>
       <x:c r="E7" s="35" t="s">
-        <x:v>362</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="F7" s="35" t="s">
-        <x:v>363</x:v>
+        <x:v>333</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="109.5" customHeight="1">
       <x:c r="A8" s="35" t="s">
-        <x:v>364</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="B8" s="35" t="s">
-        <x:v>365</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="C8" s="35" t="s">
-        <x:v>366</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="D8" s="35" t="str">
         <x:v>PIM_PERSONAL; PIM_EMP_Search_02</x:v>
       </x:c>
       <x:c r="E8" s="35" t="s">
-        <x:v>367</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="F8" s="35" t="s">
-        <x:v>368</x:v>
+        <x:v>338</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="109.5" customHeight="1">
       <x:c r="A9" s="35" t="s">
-        <x:v>369</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="B9" s="35" t="s">
-        <x:v>370</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="C9" s="35" t="s">
-        <x:v>371</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="D9" s="35" t="s">
-        <x:v>372</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="E9" s="35" t="s">
-        <x:v>373</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="F9" s="35" t="s">
-        <x:v>374</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="109.5" customHeight="1">
       <x:c r="A10" s="35" t="s">
-        <x:v>375</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="B10" s="35" t="s">
-        <x:v>376</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="C10" s="35" t="s">
-        <x:v>377</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="D10" s="35" t="str">
         <x:v>PIM_EMP_Filter_01</x:v>
       </x:c>
       <x:c r="E10" s="35" t="s">
-        <x:v>378</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="F10" s="35" t="s">
-        <x:v>379</x:v>
+        <x:v>349</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="109.5" customHeight="1">
       <x:c r="A11" s="35" t="s">
-        <x:v>380</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="B11" s="35" t="s">
-        <x:v>381</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="C11" s="35" t="s">
-        <x:v>382</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="D11" s="35" t="s">
-        <x:v>383</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="E11" s="35" t="s">
-        <x:v>384</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="F11" s="35" t="s">
-        <x:v>385</x:v>
+        <x:v>355</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="109.5" customHeight="1">
       <x:c r="A12" s="35" t="s">
-        <x:v>386</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="B12" s="35" t="s">
-        <x:v>387</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="C12" s="35" t="s">
-        <x:v>388</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="D12" s="35" t="s">
-        <x:v>389</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="E12" s="35" t="s">
-        <x:v>390</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="F12" s="35" t="s">
-        <x:v>391</x:v>
+        <x:v>361</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="109.5" customHeight="1">
       <x:c r="A13" s="35" t="s">
-        <x:v>392</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="B13" s="35" t="s">
-        <x:v>393</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="C13" s="35" t="s">
-        <x:v>394</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="D13" s="35" t="s">
-        <x:v>395</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="E13" s="35" t="s">
-        <x:v>396</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="F13" s="35" t="s">
-        <x:v>397</x:v>
+        <x:v>367</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="109.5" customHeight="1">
       <x:c r="A14" s="35" t="s">
-        <x:v>398</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="B14" s="35" t="s">
-        <x:v>399</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="C14" s="35" t="s">
-        <x:v>400</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="D14" s="35" t="s">
-        <x:v>401</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="E14" s="35" t="s">
-        <x:v>402</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="F14" s="35" t="s">
-        <x:v>403</x:v>
+        <x:v>373</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="109.5" customHeight="1">
       <x:c r="A15" s="35" t="s">
-        <x:v>404</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="B15" s="35" t="s">
-        <x:v>405</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="C15" s="35" t="s">
-        <x:v>406</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="D15" s="35" t="s">
-        <x:v>407</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E15" s="35" t="s">
-        <x:v>408</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="F15" s="35" t="s">
-        <x:v>409</x:v>
+        <x:v>379</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="109.5" customHeight="1">
       <x:c r="A16" s="35" t="s">
-        <x:v>410</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="B16" s="35" t="s">
-        <x:v>411</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="C16" s="35" t="s">
-        <x:v>412</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="D16" s="35" t="s">
-        <x:v>413</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="E16" s="35" t="s">
-        <x:v>414</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="F16" s="35" t="s">
-        <x:v>415</x:v>
+        <x:v>385</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="109.5" customHeight="1">
       <x:c r="A17" s="35" t="s">
-        <x:v>416</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="B17" s="35" t="s">
-        <x:v>417</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="C17" s="35" t="s">
-        <x:v>418</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="D17" s="35" t="str">
         <x:v>PIM_EMP_UploadPhoto_01–02</x:v>
       </x:c>
       <x:c r="E17" s="35" t="s">
-        <x:v>419</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="F17" s="35" t="s">
-        <x:v>420</x:v>
+        <x:v>390</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="109.5" customHeight="1">
       <x:c r="A18" s="35" t="s">
-        <x:v>421</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="B18" s="35" t="s">
-        <x:v>422</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="C18" s="35" t="str">
         <x:v>PDF thực. PNG hợp lệ 1.048.577 byte (1 MiB + 1 byte), có ancillary chunk; không đổi đuôi tệp.</x:v>
@@ -12358,150 +12726,150 @@
         <x:v>PIM_EMP_UploadPhoto_03–04</x:v>
       </x:c>
       <x:c r="E18" s="35" t="s">
-        <x:v>423</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="F18" s="35" t="s">
-        <x:v>424</x:v>
+        <x:v>394</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="109.5" customHeight="1">
       <x:c r="A19" s="35" t="s">
-        <x:v>425</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="B19" s="35" t="s">
-        <x:v>426</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="C19" s="35" t="s">
-        <x:v>427</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="D19" s="35" t="s">
-        <x:v>428</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="E19" s="35" t="s">
-        <x:v>429</x:v>
+        <x:v>399</x:v>
       </x:c>
       <x:c r="F19" s="35" t="s">
-        <x:v>430</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="109.5" customHeight="1">
+        <x:v>400</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="110" customHeight="1">
       <x:c r="A20" s="35" t="s">
-        <x:v>431</x:v>
-      </x:c>
-      <x:c r="B20" s="35" t="s">
-        <x:v>432</x:v>
-      </x:c>
-      <x:c r="C20" s="35" t="s">
-        <x:v>433</x:v>
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="B20" s="35" t="str">
+        <x:v>Max Attachment Size: 1048576 byte</x:v>
+      </x:c>
+      <x:c r="C20" s="35" t="str">
+        <x:v>CSV được phép; BIN (application/octet-stream) bị chặn. Tệp quá cỡ: 1.048.577 byte.</x:v>
       </x:c>
       <x:c r="D20" s="35" t="str">
         <x:v>PIM_JOB_UploadContract_02–03; các TC upload</x:v>
       </x:c>
       <x:c r="E20" s="35" t="s">
-        <x:v>434</x:v>
-      </x:c>
-      <x:c r="F20" s="35" t="s">
-        <x:v>435</x:v>
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="F20" s="35" t="str">
+        <x:v>Nguồn: evidence/executions/23130226/PIM_DETAILS_2026-10-28T03-14-37-161Z/upload-config.json</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="109.5" customHeight="1">
       <x:c r="A21" s="35" t="s">
-        <x:v>436</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="B21" s="35" t="s">
-        <x:v>437</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="C21" s="35" t="s">
-        <x:v>438</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D21" s="35" t="s">
-        <x:v>439</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="E21" s="35" t="s">
-        <x:v>440</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="F21" s="35" t="s">
-        <x:v>441</x:v>
+        <x:v>408</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="109.5" customHeight="1">
       <x:c r="A22" s="35" t="s">
-        <x:v>442</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="B22" s="35" t="s">
-        <x:v>443</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="C22" s="35" t="s">
-        <x:v>444</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="D22" s="35" t="s">
-        <x:v>445</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="E22" s="35" t="s">
-        <x:v>446</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="F22" s="35" t="s">
-        <x:v>447</x:v>
+        <x:v>414</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="109.5" customHeight="1">
       <x:c r="A23" s="35" t="s">
-        <x:v>448</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="B23" s="35" t="s">
-        <x:v>449</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="C23" s="35" t="s">
-        <x:v>450</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="D23" s="35" t="s">
-        <x:v>451</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="E23" s="35" t="s">
-        <x:v>452</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="F23" s="35" t="s">
-        <x:v>453</x:v>
+        <x:v>420</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="109.5" customHeight="1">
       <x:c r="A24" s="35" t="s">
-        <x:v>454</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="B24" s="35" t="s">
-        <x:v>455</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="C24" s="35" t="s">
-        <x:v>456</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="D24" s="35" t="s">
-        <x:v>457</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="E24" s="35" t="s">
-        <x:v>458</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="F24" s="35" t="s">
-        <x:v>459</x:v>
+        <x:v>426</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="109.5" customHeight="1">
       <x:c r="A25" s="35" t="s">
-        <x:v>460</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="B25" s="35" t="s">
-        <x:v>461</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="C25" s="35" t="s">
-        <x:v>462</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="D25" s="35" t="s">
-        <x:v>463</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="E25" s="35" t="s">
-        <x:v>464</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="F25" s="35" t="s">
-        <x:v>465</x:v>
+        <x:v>432</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15.75" customHeight="1">
@@ -12514,13 +12882,13 @@
     </x:row>
     <x:row r="27" ht="15.75" customHeight="1">
       <x:c r="A27" s="38" t="s">
-        <x:v>466</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="B27" s="38" t="s">
-        <x:v>467</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="C27" s="38" t="s">
-        <x:v>468</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="D27" s="1"/>
       <x:c r="E27" s="1"/>
@@ -12534,7 +12902,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C28" s="35" t="s">
-        <x:v>469</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="D28" s="2"/>
       <x:c r="E28" s="2"/>
@@ -12542,13 +12910,13 @@
     </x:row>
     <x:row r="29" ht="69.75" customHeight="1">
       <x:c r="A29" s="35" t="s">
-        <x:v>470</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="B29" s="35" t="s">
-        <x:v>471</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="C29" s="35" t="s">
-        <x:v>472</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="D29" s="2"/>
       <x:c r="E29" s="2"/>
@@ -12556,13 +12924,13 @@
     </x:row>
     <x:row r="30" ht="69.75" customHeight="1">
       <x:c r="A30" s="35" t="s">
-        <x:v>473</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="B30" s="35" t="s">
-        <x:v>474</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="C30" s="35" t="s">
-        <x:v>475</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="D30" s="2"/>
       <x:c r="E30" s="2"/>
@@ -12570,13 +12938,13 @@
     </x:row>
     <x:row r="31" ht="69.75" customHeight="1">
       <x:c r="A31" s="35" t="s">
-        <x:v>476</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="B31" s="35" t="s">
-        <x:v>477</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="C31" s="35" t="s">
-        <x:v>478</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D31" s="2"/>
       <x:c r="E31" s="2"/>
@@ -12587,10 +12955,10 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="B32" s="35" t="s">
-        <x:v>479</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="C32" s="35" t="s">
-        <x:v>480</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="D32" s="2"/>
       <x:c r="E32" s="2"/>
@@ -12598,13 +12966,13 @@
     </x:row>
     <x:row r="33" ht="69.75" customHeight="1">
       <x:c r="A33" s="35" t="s">
-        <x:v>481</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="B33" s="35" t="s">
-        <x:v>482</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="C33" s="35" t="s">
-        <x:v>483</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="D33" s="2"/>
       <x:c r="E33" s="2"/>
@@ -13657,7 +14025,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="3" t="s">
-        <x:v>484</x:v>
+        <x:v>451</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -13673,19 +14041,19 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B4" s="38" t="s">
-        <x:v>485</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="C4" s="38" t="s">
-        <x:v>486</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="D4" s="38" t="s">
-        <x:v>487</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="E4" s="38" t="s">
-        <x:v>488</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="F4" s="38" t="s">
-        <x:v>489</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="103.5" customHeight="1">
@@ -13693,19 +14061,19 @@
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="B5" s="35" t="s">
-        <x:v>490</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="C5" s="35" t="s">
-        <x:v>491</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="D5" s="35" t="s">
-        <x:v>492</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="E5" s="35" t="s">
-        <x:v>493</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="F5" s="35" t="str">
-        <x:v>Đã thực hiện PIM_EMP</x:v>
+        <x:v>Đã thực hiện</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="103.5" customHeight="1">
@@ -13713,19 +14081,19 @@
         <x:v>2.0</x:v>
       </x:c>
       <x:c r="B6" s="35" t="s">
-        <x:v>494</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="C6" s="35" t="str">
-        <x:v>Tạo F_DUP, F_PERSON, F_FILTER qua UI; ghi numeric employee key. Chuẩn bị JPG/PNG/PDF và PNG 1 MiB + 1 byte. F_JOB chưa tạo.</x:v>
+        <x:v>Nhân viên Personal/Job riêng, ID theo run token; PDF hợp lệ, quá giới hạn và BIN để kiểm tra upload.</x:v>
       </x:c>
       <x:c r="D6" s="35" t="s">
-        <x:v>495</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="E6" s="35" t="s">
-        <x:v>496</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="F6" s="35" t="str">
-        <x:v>Đã chuẩn bị PIM_EMP</x:v>
+        <x:v>Đã thực hiện</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="103.5" customHeight="1">
@@ -13733,19 +14101,19 @@
         <x:v>3.0</x:v>
       </x:c>
       <x:c r="B7" s="35" t="s">
-        <x:v>497</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="C7" s="35" t="str">
         <x:v>Chạy Playwright PIM_EMP, thêm assertion cho từng expected, lưu log và screenshot thật.</x:v>
       </x:c>
       <x:c r="D7" s="35" t="s">
-        <x:v>498</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="E7" s="35" t="str">
         <x:v>Playwright 1.62.1; Microsoft Edge headless.</x:v>
       </x:c>
       <x:c r="F7" s="35" t="str">
-        <x:v>Đã thực hiện PIM_EMP</x:v>
+        <x:v>Đã thực hiện</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="103.5" customHeight="1">
@@ -13753,19 +14121,19 @@
         <x:v>4.0</x:v>
       </x:c>
       <x:c r="B8" s="35" t="s">
-        <x:v>499</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="C8" s="35" t="str">
-        <x:v>Runner PIM_EMP gồm 25 case theo ID workbook, setup và cleanup riêng. PIM_PERSONAL/PIM_JOB chưa triển khai.</x:v>
+        <x:v>25 case PIM_EMP; 25 PIM_PERSONAL và 25 PIM_JOB theo ID workbook.</x:v>
       </x:c>
       <x:c r="D8" s="35" t="s">
-        <x:v>500</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="E8" s="35" t="s">
-        <x:v>501</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="F8" s="35" t="str">
-        <x:v>Đã thực hiện PIM_EMP</x:v>
+        <x:v>Đã thực hiện</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="103.5" customHeight="1">
@@ -13773,7 +14141,7 @@
         <x:v>5.0</x:v>
       </x:c>
       <x:c r="B9" s="35" t="s">
-        <x:v>502</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="C9" s="35" t="str">
         <x:v>Playwright kiểm tra validation, tìm kiếm, filter và giá trị sau Save/reload.</x:v>
@@ -13785,7 +14153,7 @@
         <x:v>Đợi phản hồi Search và UI cập nhật trước khi assertion.</x:v>
       </x:c>
       <x:c r="F9" s="35" t="str">
-        <x:v>Đã thực hiện PIM_EMP</x:v>
+        <x:v>Đã thực hiện</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="103.5" customHeight="1">
@@ -13793,19 +14161,19 @@
         <x:v>6.0</x:v>
       </x:c>
       <x:c r="B10" s="35" t="s">
-        <x:v>503</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="C10" s="35" t="str">
-        <x:v>Kiểm thử upload JPG/PNG/PDF/ảnh quá cỡ và sorting. Attachment/contract chưa chạy.</x:v>
+        <x:v>Kiểm tra attachment, giới hạn tệp; giữ/thay/xóa hợp đồng và đối chiếu nội dung PDF tải xuống.</x:v>
       </x:c>
       <x:c r="D10" s="35" t="s">
-        <x:v>504</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="E10" s="35" t="str">
         <x:v>Playwright setInputFiles; kiểm tra validation và lưu/reload.</x:v>
       </x:c>
       <x:c r="F10" s="35" t="str">
-        <x:v>Đã thực hiện PIM_EMP</x:v>
+        <x:v>Đã thực hiện</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="103.5" customHeight="1">
@@ -13813,19 +14181,19 @@
         <x:v>7.0</x:v>
       </x:c>
       <x:c r="B11" s="35" t="s">
-        <x:v>505</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="C11" s="35" t="s">
-        <x:v>506</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="D11" s="35" t="s">
-        <x:v>507</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="E11" s="35" t="str">
         <x:v>Đợi giá trị form thực, không chỉ phần tử hiện hữu.</x:v>
       </x:c>
       <x:c r="F11" s="35" t="str">
-        <x:v>Đã thực hiện PIM_EMP</x:v>
+        <x:v>Đã thực hiện</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="103.5" customHeight="1">
@@ -13833,19 +14201,19 @@
         <x:v>8.0</x:v>
       </x:c>
       <x:c r="B12" s="35" t="s">
-        <x:v>508</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="C12" s="35" t="s">
-        <x:v>509</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="D12" s="35" t="s">
-        <x:v>510</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="E12" s="35" t="str">
-        <x:v>Run PIM_EMP_20261021_04; thời gian từng case trong Note và JSON.</x:v>
+        <x:v>PIM_EMP_20261021_04; PIM_DETAILS_2026-10-28T03-06-34-596Z; PIM_DETAILS_2026-10-28T03-14-37-161Z</x:v>
       </x:c>
       <x:c r="F12" s="35" t="str">
-        <x:v>Đã thực hiện PIM_EMP</x:v>
+        <x:v>Đã thực hiện</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="103.5" customHeight="1">
@@ -13853,19 +14221,19 @@
         <x:v>9.0</x:v>
       </x:c>
       <x:c r="B13" s="35" t="s">
-        <x:v>511</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="C13" s="35" t="s">
-        <x:v>512</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="D13" s="35" t="s">
-        <x:v>513</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="E13" s="35" t="s">
-        <x:v>514</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="F13" s="35" t="str">
-        <x:v>Xem log cleanup</x:v>
+        <x:v>Đã dọn dữ liệu</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="103.5" customHeight="1">
@@ -13873,16 +14241,16 @@
         <x:v>10.0</x:v>
       </x:c>
       <x:c r="B14" s="35" t="s">
-        <x:v>515</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="C14" s="35" t="s">
-        <x:v>516</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="D14" s="35" t="s">
-        <x:v>517</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E14" s="35" t="s">
-        <x:v>518</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="F14" s="35" t="str">
         <x:v>Thiết kế đã rà soát</x:v>
@@ -13906,7 +14274,7 @@
     </x:row>
     <x:row r="17" ht="44" customHeight="1">
       <x:c r="A17" s="2" t="str">
-        <x:v>PIM_EMP đã chạy bằng Playwright. Hai chức năng PIM_PERSONAL/PIM_JOB chưa chạy, giữ Untested. ID dùng Module_Action_XX; số thứ tự bắt đầu từ 01 trong từng nhóm hành động.</x:v>
+        <x:v>Đã chạy 75 case của ba chức năng PIM. Kết quả từng case và các lần chạy nằm trong evidence/executions/23130226/.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -14938,7 +15306,7 @@
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
       <x:c r="B1" s="3" t="s">
-        <x:v>519</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -14981,29 +15349,29 @@
       <x:c r="H4" s="39"/>
       <x:c r="I4" s="39"/>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="65" customHeight="1">
       <x:c r="B5" s="35" t="s">
-        <x:v>520</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="C5" s="39"/>
       <x:c r="D5" s="46" t="str">
-        <x:v>PIM_EMP_20261021_04</x:v>
+        <x:v>PIM_EMP_20261021_04; PIM_DETAILS_2026-10-28T03-06-34-596Z; PIM_DETAILS_2026-10-28T03-14-37-161Z</x:v>
       </x:c>
       <x:c r="E5" s="36"/>
       <x:c r="F5" s="36"/>
       <x:c r="G5" s="50" t="d">
-        <x:v>2026-10-21T10:26:20.547Z</x:v>
+        <x:v>2026-10-28T03:20:14.908Z</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="36"/>
     </x:row>
     <x:row r="6">
       <x:c r="B6" s="35" t="s">
-        <x:v>521</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="C6" s="39"/>
       <x:c r="D6" s="46" t="str">
-        <x:v>Playwright / Microsoft Edge 155.0.4283.62 (headless)</x:v>
+        <x:v>Playwright / Edge 155.0.4283.62 (EMP); 156.0.4314.50 (PERSONAL/JOB)</x:v>
       </x:c>
       <x:c r="E6" s="36"/>
       <x:c r="F6" s="36"/>
@@ -15054,7 +15422,7 @@
         <x:v>108</x:v>
       </x:c>
       <x:c r="I9" s="38" t="s">
-        <x:v>522</x:v>
+        <x:v>489</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
@@ -15098,7 +15466,7 @@
       </x:c>
       <x:c r="D11" s="35" t="n">
         <x:f>PIM_PERSONAL!A6</x:f>
-        <x:v>0</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E11" s="35" t="n">
         <x:f>PIM_PERSONAL!B6</x:f>
@@ -15106,7 +15474,7 @@
       </x:c>
       <x:c r="F11" s="35" t="n">
         <x:f>PIM_PERSONAL!C6</x:f>
-        <x:v>25</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="35" t="n">
         <x:f>PIM_PERSONAL!D6</x:f>
@@ -15130,7 +15498,7 @@
       </x:c>
       <x:c r="D12" s="35" t="n">
         <x:f>PIM_JOB!A6</x:f>
-        <x:v>0</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E12" s="35" t="n">
         <x:f>PIM_JOB!B6</x:f>
@@ -15138,7 +15506,7 @@
       </x:c>
       <x:c r="F12" s="35" t="n">
         <x:f>PIM_JOB!C6</x:f>
-        <x:v>25</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="35" t="n">
         <x:f>PIM_JOB!D6</x:f>
@@ -15165,12 +15533,12 @@
     </x:row>
     <x:row r="14">
       <x:c r="B14" s="47" t="s">
-        <x:v>522</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="C14" s="36"/>
       <x:c r="D14" s="47" t="n">
         <x:f t="shared" ref="D14:I14" si="1">SUM(D10:D12)</x:f>
-        <x:v>23</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="E14" s="47" t="n">
         <x:f t="shared" si="1">SUM(E10:E12)</x:f>
@@ -15178,7 +15546,7 @@
       </x:c>
       <x:c r="F14" s="47" t="n">
         <x:f t="shared" si="1">SUM(F10:F12)</x:f>
-        <x:v>50</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="47" t="n">
         <x:f t="shared" si="1">SUM(G10:G12)</x:f>
@@ -15215,13 +15583,13 @@
     </x:row>
     <x:row r="17">
       <x:c r="B17" s="35" t="s">
-        <x:v>523</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="C17" s="39"/>
       <x:c r="D17" s="39"/>
       <x:c r="E17" s="48" t="n">
         <x:f>IF(I14=0,"",(D14+E14)/I14)</x:f>
-        <x:v>0.30666666666666664</x:v>
+        <x:v>0.9733333333333334</x:v>
       </x:c>
       <x:c r="F17" s="39"/>
       <x:c r="G17" s="2"/>
@@ -15230,7 +15598,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="B18" s="35" t="s">
-        <x:v>524</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="C18" s="39"/>
       <x:c r="D18" s="39"/>
@@ -15255,7 +15623,7 @@
     </x:row>
     <x:row r="20" ht="39.75" customHeight="1">
       <x:c r="B20" s="2" t="s">
-        <x:v>525</x:v>
+        <x:v>492</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
@@ -15270,7 +15638,7 @@
     </x:row>
     <x:row r="22" ht="65" customHeight="1">
       <x:c r="B22" s="2" t="str">
-        <x:v>Kết quả PIM_EMP: 23 Passed, 0 Failed, 2 Blocked. PIM_PERSONAL/PIM_JOB: 50 Untested. Log và ảnh: evidence/executions/23130226/PIM_EMP_20261021_04/. Các run trước dùng chẩn đoán script, không cộng dồn vào report.</x:v>
+        <x:v>PIM_EMP: 23 Passed, 2 Blocked. PIM_PERSONAL/PIM_JOB: 50 Passed, 0 Failed, 0 Blocked. Lấy kết quả mới nhất theo Case ID; đường dẫn log/ảnh tại cột Note.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">

</xml_diff>